<commit_message>
Carregado dados de Dez/2025
</commit_message>
<xml_diff>
--- a/upload/mp_setor.xlsx
+++ b/upload/mp_setor.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\x17954399\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\m10428324\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12180"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12300"/>
   </bookViews>
   <sheets>
     <sheet name="Export" sheetId="1" r:id="rId1"/>
@@ -21110,7 +21110,7 @@
         <v>81</v>
       </c>
       <c r="E1206">
-        <v>7.3508771929824563</v>
+        <v>7.2241379310344831</v>
       </c>
     </row>
     <row r="1207" spans="1:5">
@@ -21161,7 +21161,7 @@
         <v>83</v>
       </c>
       <c r="E1209">
-        <v>0.87573964497041423</v>
+        <v>0.87058823529411766</v>
       </c>
     </row>
     <row r="1210" spans="1:5">

</xml_diff>